<commit_message>
Updated UALR Net Spreadsheet to include Log
</commit_message>
<xml_diff>
--- a/DIY_Hotspot/UALR_Net_List_Spreadsheet_Central_Time.xlsx
+++ b/DIY_Hotspot/UALR_Net_List_Spreadsheet_Central_Time.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ad1f42790ad99ab6/Documents/Repositories/D-Star/DIY_Hotspot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_86925A58680A957D1B068367EBB309C97348CDB1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF9E9FAF-7011-44CB-8C9E-8014EF5B8735}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="11_86925A58680A957D1B068367EBB309C97348CDB1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BCACC21A-8F34-45C3-95C0-900487EBCBC6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Source" sheetId="1" r:id="rId1"/>
+    <sheet name="Log and Notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$M$254</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$M$252</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Source!$A$2:$M$254</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Source!$A$1:$M$252</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1342" uniqueCount="465">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1373" uniqueCount="467">
   <si>
     <t>Echolink and D Star Net Listings</t>
   </si>
@@ -1754,6 +1755,13 @@
   </si>
   <si>
     <t>Young Operators Digital Voice Net</t>
+  </si>
+  <si>
+    <t>Plan:  5/3/25</t>
+  </si>
+  <si>
+    <t>Memphis Chat Room
+5/2/25</t>
   </si>
 </sst>
 </file>
@@ -1926,7 +1934,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1983,6 +1991,10 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2384,6 +2396,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -2653,7 +2669,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="16.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>24</v>
       </c>
@@ -2775,7 +2791,7 @@
       </c>
       <c r="M9" s="13"/>
     </row>
-    <row r="10" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A10" s="10" t="s">
         <v>35</v>
       </c>
@@ -2802,7 +2818,7 @@
       </c>
       <c r="M10" s="16"/>
     </row>
-    <row r="11" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A11" s="10" t="s">
         <v>37</v>
       </c>
@@ -2825,7 +2841,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A12" s="10" t="s">
         <v>40</v>
       </c>
@@ -2846,7 +2862,7 @@
       </c>
       <c r="M12" s="13"/>
     </row>
-    <row r="13" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A13" s="10" t="s">
         <v>42</v>
       </c>
@@ -2867,7 +2883,7 @@
       </c>
       <c r="M13" s="13"/>
     </row>
-    <row r="14" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A14" s="10" t="s">
         <v>43</v>
       </c>
@@ -2888,7 +2904,7 @@
       </c>
       <c r="M14" s="13"/>
     </row>
-    <row r="15" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A15" s="10" t="s">
         <v>45</v>
       </c>
@@ -2932,7 +2948,7 @@
       </c>
       <c r="M16" s="13"/>
     </row>
-    <row r="17" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A17" s="10" t="s">
         <v>50</v>
       </c>
@@ -2982,7 +2998,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" ht="15" x14ac:dyDescent="0.35">
       <c r="A19" s="10" t="s">
         <v>53</v>
       </c>
@@ -3086,7 +3102,7 @@
       </c>
       <c r="M22" s="13"/>
     </row>
-    <row r="23" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A23" s="10" t="s">
         <v>62</v>
       </c>
@@ -3107,7 +3123,7 @@
       </c>
       <c r="M23" s="13"/>
     </row>
-    <row r="24" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A24" s="10" t="s">
         <v>63</v>
       </c>
@@ -3130,7 +3146,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A25" s="10" t="s">
         <v>65</v>
       </c>
@@ -3197,7 +3213,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A28" s="10" t="s">
         <v>72</v>
       </c>
@@ -3285,7 +3301,7 @@
       </c>
       <c r="M30" s="13"/>
     </row>
-    <row r="31" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A31" s="10" t="s">
         <v>78</v>
       </c>
@@ -3388,7 +3404,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A34" s="10" t="s">
         <v>83</v>
       </c>
@@ -3457,7 +3473,7 @@
       </c>
       <c r="M36" s="13"/>
     </row>
-    <row r="37" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A37" s="10" t="s">
         <v>88</v>
       </c>
@@ -3504,7 +3520,7 @@
       </c>
       <c r="M38" s="13"/>
     </row>
-    <row r="39" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A39" s="10" t="s">
         <v>92</v>
       </c>
@@ -3567,7 +3583,7 @@
       </c>
       <c r="M41" s="13"/>
     </row>
-    <row r="42" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A42" s="10" t="s">
         <v>98</v>
       </c>
@@ -3636,7 +3652,7 @@
       </c>
       <c r="M44" s="18"/>
     </row>
-    <row r="45" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A45" s="10" t="s">
         <v>103</v>
       </c>
@@ -3703,7 +3719,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A47" s="10" t="s">
         <v>107</v>
       </c>
@@ -3747,7 +3763,7 @@
       </c>
       <c r="M48" s="13"/>
     </row>
-    <row r="49" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A49" s="10" t="s">
         <v>112</v>
       </c>
@@ -3810,7 +3826,7 @@
       </c>
       <c r="M51" s="13"/>
     </row>
-    <row r="52" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A52" s="10" t="s">
         <v>117</v>
       </c>
@@ -3889,7 +3905,7 @@
       </c>
       <c r="M54" s="13"/>
     </row>
-    <row r="55" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A55" s="10" t="s">
         <v>122</v>
       </c>
@@ -3912,7 +3928,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="56" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A56" s="10" t="s">
         <v>125</v>
       </c>
@@ -4016,7 +4032,7 @@
       </c>
       <c r="M59" s="13"/>
     </row>
-    <row r="60" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A60" s="10" t="s">
         <v>133</v>
       </c>
@@ -4062,7 +4078,7 @@
       </c>
       <c r="M61" s="13"/>
     </row>
-    <row r="62" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A62" s="10" t="s">
         <v>138</v>
       </c>
@@ -4084,7 +4100,7 @@
       </c>
       <c r="M62" s="13"/>
     </row>
-    <row r="63" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A63" s="10" t="s">
         <v>139</v>
       </c>
@@ -4111,7 +4127,7 @@
       </c>
       <c r="M63" s="18"/>
     </row>
-    <row r="64" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A64" s="10" t="s">
         <v>141</v>
       </c>
@@ -4137,7 +4153,7 @@
       </c>
       <c r="M64" s="18"/>
     </row>
-    <row r="65" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A65" s="10" t="s">
         <v>142</v>
       </c>
@@ -4181,7 +4197,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A67" s="10" t="s">
         <v>145</v>
       </c>
@@ -4233,7 +4249,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="69" spans="1:13" ht="15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:13" ht="15" x14ac:dyDescent="0.35">
       <c r="A69" s="10" t="s">
         <v>151</v>
       </c>
@@ -4321,7 +4337,7 @@
       </c>
       <c r="M72" s="13"/>
     </row>
-    <row r="73" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A73" s="10" t="s">
         <v>161</v>
       </c>
@@ -4344,7 +4360,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="74" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A74" s="10" t="s">
         <v>164</v>
       </c>
@@ -4367,7 +4383,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="75" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A75" s="10" t="s">
         <v>166</v>
       </c>
@@ -4514,7 +4530,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="80" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A80" s="10" t="s">
         <v>175</v>
       </c>
@@ -4582,7 +4598,7 @@
       </c>
       <c r="M82" s="13"/>
     </row>
-    <row r="83" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A83" s="10" t="s">
         <v>181</v>
       </c>
@@ -4605,7 +4621,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="84" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A84" s="10" t="s">
         <v>183</v>
       </c>
@@ -4629,7 +4645,7 @@
       </c>
       <c r="M84" s="13"/>
     </row>
-    <row r="85" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A85" s="10" t="s">
         <v>185</v>
       </c>
@@ -4650,7 +4666,7 @@
       </c>
       <c r="M85" s="13"/>
     </row>
-    <row r="86" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A86" s="10" t="s">
         <v>187</v>
       </c>
@@ -4671,7 +4687,7 @@
       </c>
       <c r="M86" s="13"/>
     </row>
-    <row r="87" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A87" s="10" t="s">
         <v>188</v>
       </c>
@@ -4731,7 +4747,7 @@
       </c>
       <c r="M88" s="13"/>
     </row>
-    <row r="89" spans="1:13" s="14" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:13" s="14" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A89" s="10" t="s">
         <v>191</v>
       </c>
@@ -4758,7 +4774,7 @@
       </c>
       <c r="M89" s="13"/>
     </row>
-    <row r="90" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A90" s="10" t="s">
         <v>192</v>
       </c>
@@ -4866,7 +4882,7 @@
       </c>
       <c r="M93" s="13"/>
     </row>
-    <row r="94" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A94" s="10" t="s">
         <v>201</v>
       </c>
@@ -4996,7 +5012,7 @@
       </c>
       <c r="M99" s="13"/>
     </row>
-    <row r="100" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A100" s="10" t="s">
         <v>212</v>
       </c>
@@ -5087,7 +5103,7 @@
       </c>
       <c r="M103" s="13"/>
     </row>
-    <row r="104" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A104" s="10" t="s">
         <v>219</v>
       </c>
@@ -5108,7 +5124,7 @@
       </c>
       <c r="M104" s="13"/>
     </row>
-    <row r="105" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A105" s="10" t="s">
         <v>220</v>
       </c>
@@ -5131,7 +5147,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="106" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A106" s="10" t="s">
         <v>223</v>
       </c>
@@ -5226,7 +5242,7 @@
       </c>
       <c r="M109" s="13"/>
     </row>
-    <row r="110" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A110" s="10" t="s">
         <v>229</v>
       </c>
@@ -5280,7 +5296,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="112" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A112" s="10" t="s">
         <v>234</v>
       </c>
@@ -5347,7 +5363,7 @@
       </c>
       <c r="M114" s="13"/>
     </row>
-    <row r="115" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A115" s="10" t="s">
         <v>238</v>
       </c>
@@ -5368,7 +5384,7 @@
       </c>
       <c r="M115" s="13"/>
     </row>
-    <row r="116" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A116" s="10" t="s">
         <v>239</v>
       </c>
@@ -5389,7 +5405,7 @@
       </c>
       <c r="M116" s="13"/>
     </row>
-    <row r="117" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A117" s="14" t="s">
         <v>240</v>
       </c>
@@ -5412,7 +5428,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="118" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A118" s="10" t="s">
         <v>243</v>
       </c>
@@ -5462,7 +5478,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="120" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A120" s="10" t="s">
         <v>248</v>
       </c>
@@ -5506,7 +5522,7 @@
       </c>
       <c r="M121" s="13"/>
     </row>
-    <row r="122" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A122" s="10" t="s">
         <v>252</v>
       </c>
@@ -5527,7 +5543,7 @@
       </c>
       <c r="M122" s="13"/>
     </row>
-    <row r="123" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A123" s="10" t="s">
         <v>254</v>
       </c>
@@ -5550,7 +5566,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="124" spans="1:14" s="14" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:14" s="14" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A124" s="10" t="s">
         <v>257</v>
       </c>
@@ -5599,7 +5615,7 @@
       </c>
       <c r="M125" s="13"/>
     </row>
-    <row r="126" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A126" s="10" t="s">
         <v>260</v>
       </c>
@@ -5643,7 +5659,7 @@
       </c>
       <c r="M127" s="13"/>
     </row>
-    <row r="128" spans="1:14" ht="15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:14" ht="15" x14ac:dyDescent="0.35">
       <c r="A128" s="10" t="s">
         <v>264</v>
       </c>
@@ -5690,7 +5706,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="130" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A130" s="10" t="s">
         <v>269</v>
       </c>
@@ -5761,7 +5777,7 @@
       </c>
       <c r="M132" s="13"/>
     </row>
-    <row r="133" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A133" s="10" t="s">
         <v>276</v>
       </c>
@@ -6005,7 +6021,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="140" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A140" s="10" t="s">
         <v>285</v>
       </c>
@@ -6069,7 +6085,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="142" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A142" s="10" t="s">
         <v>289</v>
       </c>
@@ -6181,7 +6197,7 @@
       </c>
       <c r="M145" s="18"/>
     </row>
-    <row r="146" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A146" s="10" t="s">
         <v>296</v>
       </c>
@@ -6207,7 +6223,7 @@
       </c>
       <c r="M146" s="18"/>
     </row>
-    <row r="147" spans="1:13" s="10" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:13" s="10" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A147" s="10" t="s">
         <v>297</v>
       </c>
@@ -6259,7 +6275,7 @@
       </c>
       <c r="M148" s="18"/>
     </row>
-    <row r="149" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A149" s="10" t="s">
         <v>300</v>
       </c>
@@ -6313,7 +6329,7 @@
       </c>
       <c r="M150" s="18"/>
     </row>
-    <row r="151" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A151" s="10" t="s">
         <v>303</v>
       </c>
@@ -6521,7 +6537,7 @@
       </c>
       <c r="M159" s="13"/>
     </row>
-    <row r="160" spans="1:13" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A160" s="10" t="s">
         <v>319</v>
       </c>
@@ -6689,7 +6705,7 @@
       </c>
       <c r="M166" s="13"/>
     </row>
-    <row r="167" spans="1:14" ht="15" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:14" ht="15" x14ac:dyDescent="0.35">
       <c r="A167" s="10" t="s">
         <v>330</v>
       </c>
@@ -6751,7 +6767,7 @@
       </c>
       <c r="M168" s="13"/>
     </row>
-    <row r="169" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A169" s="10" t="s">
         <v>335</v>
       </c>
@@ -6822,7 +6838,7 @@
       </c>
       <c r="M171" s="13"/>
     </row>
-    <row r="172" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A172" s="10" t="s">
         <v>339</v>
       </c>
@@ -6843,7 +6859,7 @@
       </c>
       <c r="M172" s="13"/>
     </row>
-    <row r="173" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A173" s="10" t="s">
         <v>340</v>
       </c>
@@ -6969,7 +6985,7 @@
       </c>
       <c r="M178" s="13"/>
     </row>
-    <row r="179" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A179" s="10" t="s">
         <v>352</v>
       </c>
@@ -7072,7 +7088,7 @@
       </c>
       <c r="M181" s="13"/>
     </row>
-    <row r="182" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A182" s="10" t="s">
         <v>356</v>
       </c>
@@ -7128,7 +7144,7 @@
       </c>
       <c r="M183" s="13"/>
     </row>
-    <row r="184" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A184" s="10" t="s">
         <v>359</v>
       </c>
@@ -7312,7 +7328,7 @@
       </c>
       <c r="M189" s="13"/>
     </row>
-    <row r="190" spans="1:21" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:21" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A190" s="10" t="s">
         <v>366</v>
       </c>
@@ -7520,7 +7536,7 @@
       </c>
       <c r="M197" s="13"/>
     </row>
-    <row r="198" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A198" s="10" t="s">
         <v>377</v>
       </c>
@@ -7570,7 +7586,7 @@
       </c>
       <c r="M199" s="13"/>
     </row>
-    <row r="200" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A200" s="10" t="s">
         <v>380</v>
       </c>
@@ -7770,7 +7786,7 @@
       <c r="M207" s="13"/>
       <c r="N207" s="14"/>
     </row>
-    <row r="208" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A208" s="10" t="s">
         <v>394</v>
       </c>
@@ -7811,7 +7827,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="209" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A209" s="10" t="s">
         <v>395</v>
       </c>
@@ -7862,7 +7878,7 @@
       <c r="M210" s="13"/>
       <c r="N210"/>
     </row>
-    <row r="211" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A211" s="10" t="s">
         <v>399</v>
       </c>
@@ -7951,7 +7967,7 @@
       <c r="M214" s="13"/>
       <c r="N214" s="14"/>
     </row>
-    <row r="215" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A215" s="10" t="s">
         <v>406</v>
       </c>
@@ -8257,7 +8273,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="227" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A227" s="10" t="s">
         <v>423</v>
       </c>
@@ -8280,7 +8296,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="228" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A228" s="10" t="s">
         <v>425</v>
       </c>
@@ -8345,7 +8361,7 @@
       </c>
       <c r="M230" s="13"/>
     </row>
-    <row r="231" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A231" s="10" t="s">
         <v>429</v>
       </c>
@@ -8451,7 +8467,7 @@
       </c>
       <c r="M234" s="13"/>
     </row>
-    <row r="235" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A235" s="10" t="s">
         <v>437</v>
       </c>
@@ -8501,7 +8517,7 @@
       </c>
       <c r="M236" s="13"/>
     </row>
-    <row r="237" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A237" s="10" t="s">
         <v>441</v>
       </c>
@@ -8566,7 +8582,7 @@
       </c>
       <c r="M239" s="13"/>
     </row>
-    <row r="240" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A240" s="10" t="s">
         <v>444</v>
       </c>
@@ -8616,7 +8632,7 @@
       <c r="M241" s="13"/>
       <c r="N241" s="21"/>
     </row>
-    <row r="242" spans="1:14" s="21" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:14" s="21" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A242" s="10" t="s">
         <v>447</v>
       </c>
@@ -8686,7 +8702,7 @@
       </c>
       <c r="M244" s="13"/>
     </row>
-    <row r="245" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A245" s="10" t="s">
         <v>452</v>
       </c>
@@ -8707,7 +8723,7 @@
       </c>
       <c r="M245" s="13"/>
     </row>
-    <row r="246" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A246" s="10" t="s">
         <v>453</v>
       </c>
@@ -8871,7 +8887,7 @@
       </c>
       <c r="N250" s="21"/>
     </row>
-    <row r="251" spans="1:14" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A251" s="10" t="s">
         <v>459</v>
       </c>
@@ -8961,7 +8977,7 @@
       </c>
       <c r="N253" s="21"/>
     </row>
-    <row r="254" spans="1:14" s="14" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:14" s="14" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A254" s="10" t="s">
         <v>464</v>
       </c>
@@ -8993,11 +9009,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A2:M254" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="6">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
     <filterColumn colId="10">
       <filters>
         <filter val="D-Star"/>
@@ -9012,4 +9023,182 @@
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB0AF945-7576-4D74-91AB-654BB6BB7386}">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="27.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="3.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="3.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" s="5"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="J2" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="M2" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="39.5" x14ac:dyDescent="0.35">
+      <c r="A4" s="10" t="s">
+        <v>220</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="12">
+        <v>0.85416666666666696</v>
+      </c>
+      <c r="J4" s="12">
+        <v>6.25E-2</v>
+      </c>
+      <c r="K4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L4" t="s">
+        <v>221</v>
+      </c>
+      <c r="M4" s="27" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A5" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" s="1"/>
+      <c r="I5" s="12">
+        <v>0.79166666666666696</v>
+      </c>
+      <c r="J5" s="12">
+        <v>0</v>
+      </c>
+      <c r="K5" t="s">
+        <v>25</v>
+      </c>
+      <c r="L5" t="s">
+        <v>313</v>
+      </c>
+      <c r="M5" s="26">
+        <v>45779</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A7" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I7" s="12">
+        <v>0.85416666666666696</v>
+      </c>
+      <c r="J7" s="12">
+        <v>6.25E-2</v>
+      </c>
+      <c r="K7" t="s">
+        <v>25</v>
+      </c>
+      <c r="L7" t="s">
+        <v>64</v>
+      </c>
+      <c r="M7" t="s">
+        <v>465</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B1" r:id="rId1" xr:uid="{3BA3D2D3-6CB1-4B56-AE32-0001FAB195BC}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updating Config and Image Information Files
</commit_message>
<xml_diff>
--- a/DIY_Hotspot/UALR_Net_List_Spreadsheet_Central_Time.xlsx
+++ b/DIY_Hotspot/UALR_Net_List_Spreadsheet_Central_Time.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ad1f42790ad99ab6/Documents/Repositories/D-Star/DIY_Hotspot/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="29" documentId="11_86925A58680A957D1B068367EBB309C97348CDB1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C25F1ADF-ED14-469F-8F39-FAA42F49893E}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="11_86925A58680A957D1B068367EBB309C97348CDB1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0668BE8-0E53-4EF9-823C-1A795A55A4BD}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2393,6 +2393,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>

</xml_diff>